<commit_message>
fix(security): final review fixes - busy-path log, LENGTH_REQUIRED text, extra tests, finding labels
</commit_message>
<xml_diff>
--- a/Reports/Assessment-Stage-C-Test-Report.xlsx
+++ b/Reports/Assessment-Stage-C-Test-Report.xlsx
@@ -455,7 +455,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Full suite on branch assessment-c-security (Tasks 1 to 10; Task 11, enforcing the script-src policy, is NOT done) plus the docs commit, run 30 October 2026 on the Docker test database. Delivers: deleting an account asks for the password (4), a cookie write without Origin is refused and private answers are never cached (28 a, c), list reads write nothing and show a lapsed item as expired while a lapsed proposal still reopens at once when someone acts (28 b), profile, service, reference, name and photo-description texts refuse contact details (28 d), chat sending limited to 30 messages in 10 minutes (9, code part), blocked contact text deleted after 90 days with a cron duration and a complete env example (28 e), uploads cut off while being read and a 25 megapixel limit (12), HSTS with subdomains and a report-only script-src trial (14, partly), the back office returns no payment or tax fields and checks user ids (29, 10). No migration; kando-dev had its row-level-security file re-applied (still 0023); kando-main is untouched at 0021. Nothing was seen on a phone.</t>
+          <t>Full suite on branch assessment-c-security (Tasks 1 to 10; Task 11, enforcing the script-src policy, is NOT done) plus the docs commit, run 30 October 2026 on the Docker test database. Delivers: deleting an account asks for the password (4), a cookie write without Origin is refused and private answers are never cached (28 a, c), list reads write nothing and show a lapsed item as expired while a lapsed proposal still reopens at once when someone acts (28 b), profile, service, reference, name and photo-description texts refuse contact details (10), chat sending limited to 30 messages in 10 minutes (9, code part), blocked contact text deleted after 90 days with a cron duration and a complete env example (28 d, 29), uploads cut off while being read and a 25 megapixel limit (12), HSTS with subdomains and a report-only script-src trial (14, partly), the back office returns no payment or tax fields and checks user ids (11, 28 e). No migration; kando-dev had its row-level-security file re-applied (still 0023); kando-main is untouched at 0021. Nothing was seen on a phone.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -705,7 +705,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>rules.test.ts (bookingShownStatus); timers.int.spec.ts (a lapsed request reads expired and writes nothing, a new request is accepted; a list read writes nothing); bookings.int.spec.ts; requests-quotes specs (reopen on act)</t>
+          <t>rules.test.ts (bookingShownStatus); timers.int.spec.ts (a lapsed request reads expired and writes nothing, a new request is accepted; a list read writes nothing); bookings.int.spec.ts; timers.int.spec.ts (a lapsed proposal reopens its request and quote when someone acts)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -717,7 +717,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>28d - profile, service, reference, name and photo texts could carry contact details</t>
+          <t>10 - profile, service, reference, name and photo texts could carry contact details</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>contact-public.int.spec.ts (profile, service add and update, reference add and update, name, photo alt; no attempt recorded and no flag after many refusals); mobile use-session.test.ts (refused sign-up name dropped)</t>
+          <t>contact-public.int.spec.ts (profile, service add and update, reference add and update, name, photo alt (422, no stored object); no attempt recorded and no flag after many refusals); mobile use-session.test.ts (refused sign-up name dropped)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -761,7 +761,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>28e - blocked contact text kept forever, cron without duration, incomplete env example</t>
+          <t>28d and 29 - blocked contact text kept forever (28d); cron without duration, incomplete env example (29)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>29 and 10 - back office provider read returned payment and tax fields; user id not checked</t>
+          <t>11 and 28e - back office provider read returned payment and tax fields (11); user id not checked (28e)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">

</xml_diff>